<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@8f6d493c55531e0db0f05c65a2d8483cdf56d438 🚀
</commit_message>
<xml_diff>
--- a/epic-rolcode.xlsx
+++ b/epic-rolcode.xlsx
@@ -8,12 +8,13 @@
   <sheets>
     <sheet name="Metadata" r:id="rId3" sheetId="1"/>
     <sheet name="Mapping Table 0" r:id="rId4" sheetId="2"/>
+    <sheet name="Mapping Table 1" r:id="rId5" sheetId="3"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="41">
   <si>
     <t>Property</t>
   </si>
@@ -42,7 +43,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Epic Practitioner.qualifier to SNOMED-CT rolcode Mapping</t>
+    <t>Epic qualifier &amp; role to SNOMED-CT rolcode Mapping</t>
   </si>
   <si>
     <t>Status</t>
@@ -60,7 +61,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-07-22T08:52:45+00:00</t>
+    <t>2024-07-22T09:01:17+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -130,6 +131,12 @@
   </si>
   <si>
     <t>Medical doctor</t>
+  </si>
+  <si>
+    <t>urn:oid:1.2.840.114350.1.13.485.3.7.10.836982.1040</t>
+  </si>
+  <si>
+    <t>1</t>
   </si>
 </sst>
 </file>
@@ -450,4 +457,65 @@
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="B1" t="s" s="1">
+        <v>28</v>
+      </c>
+      <c r="C1" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="D1" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="E1" t="s" s="1">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="2">
+        <v>39</v>
+      </c>
+      <c r="B2" t="s" s="2">
+        <v>32</v>
+      </c>
+      <c r="C2" t="s" s="2">
+        <v>32</v>
+      </c>
+      <c r="D2" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="E2" t="s" s="2">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B3" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="C3" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="D3" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="E3" t="s" s="2">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@2dd4b9db12e03ac3e73a78b0f6c80dd7079a3d19 🚀
</commit_message>
<xml_diff>
--- a/epic-rolcode.xlsx
+++ b/epic-rolcode.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="48">
   <si>
     <t>Property</t>
   </si>
@@ -61,7 +61,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-07-22T09:01:17+00:00</t>
+    <t>2024-07-22T09:17:40+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -137,6 +137,27 @@
   </si>
   <si>
     <t>1</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>Physician assistant</t>
+  </si>
+  <si>
+    <t>449161006</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>Verpleegkundige specialist</t>
+  </si>
+  <si>
+    <t>224571005</t>
+  </si>
+  <si>
+    <t>Nurse practitioner</t>
   </si>
 </sst>
 </file>
@@ -461,7 +482,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -515,6 +536,40 @@
         <v>38</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="B4" t="s" s="2">
+        <v>42</v>
+      </c>
+      <c r="C4" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="D4" t="s" s="2">
+        <v>43</v>
+      </c>
+      <c r="E4" t="s" s="2">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="2">
+        <v>44</v>
+      </c>
+      <c r="B5" t="s" s="2">
+        <v>45</v>
+      </c>
+      <c r="C5" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="D5" t="s" s="2">
+        <v>46</v>
+      </c>
+      <c r="E5" t="s" s="2">
+        <v>47</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@7e5199e7e7629e08e0055f3f8e9256aebf18b4fe 🚀
</commit_message>
<xml_diff>
--- a/epic-rolcode.xlsx
+++ b/epic-rolcode.xlsx
@@ -8,13 +8,12 @@
   <sheets>
     <sheet name="Metadata" r:id="rId3" sheetId="1"/>
     <sheet name="Mapping Table 0" r:id="rId4" sheetId="2"/>
-    <sheet name="Mapping Table 1" r:id="rId5" sheetId="3"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="46">
   <si>
     <t>Property</t>
   </si>
@@ -43,7 +42,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Epic qualifier &amp; role to SNOMED-CT rolcode Mapping</t>
+    <t>Epic qualifier &amp; role to SNOMED-CT Mapping</t>
   </si>
   <si>
     <t>Status</t>
@@ -61,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-07-22T09:17:40+00:00</t>
+    <t>2024-07-22T09:30:07+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -88,7 +87,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Deze ConceptMap representeert de mapping tussen de Epic Practitioner.qualifier SER#6000 naar een SNOMED-CT rolcode.</t>
+    <t>Deze ConceptMap representeert de mapping tussen de Epic Practitioner.qualifier SER#6000 naar een SNOMED-CT code.</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -109,7 +108,7 @@
     <t>Target</t>
   </si>
   <si>
-    <t>urn:oid:1.2.840.114350.1.13.485.3.7.4.836982.6000</t>
+    <t>urn:oid:1.2.840.114350.1.13.485.3.7.10.836982.1040</t>
   </si>
   <si>
     <t/>
@@ -118,7 +117,7 @@
     <t>http://snomed.info/sct</t>
   </si>
   <si>
-    <t>11</t>
+    <t>1</t>
   </si>
   <si>
     <t>Arts</t>
@@ -131,12 +130,6 @@
   </si>
   <si>
     <t>Medical doctor</t>
-  </si>
-  <si>
-    <t>urn:oid:1.2.840.114350.1.13.485.3.7.10.836982.1040</t>
-  </si>
-  <si>
-    <t>1</t>
   </si>
   <si>
     <t>6</t>
@@ -421,67 +414,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="1">
-        <v>27</v>
-      </c>
-      <c r="B1" t="s" s="1">
-        <v>28</v>
-      </c>
-      <c r="C1" t="s" s="1">
-        <v>29</v>
-      </c>
-      <c r="D1" t="s" s="1">
-        <v>30</v>
-      </c>
-      <c r="E1" t="s" s="1">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="2">
-        <v>31</v>
-      </c>
-      <c r="B2" t="s" s="2">
-        <v>32</v>
-      </c>
-      <c r="C2" t="s" s="2">
-        <v>32</v>
-      </c>
-      <c r="D2" t="s" s="2">
-        <v>33</v>
-      </c>
-      <c r="E2" t="s" s="2">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="2">
-        <v>34</v>
-      </c>
-      <c r="B3" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="C3" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="D3" t="s" s="2">
-        <v>37</v>
-      </c>
-      <c r="E3" t="s" s="2">
-        <v>38</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
@@ -504,7 +436,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s" s="2">
         <v>32</v>
@@ -521,7 +453,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B3" t="s" s="2">
         <v>35</v>
@@ -538,36 +470,36 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C4" t="s" s="2">
         <v>36</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C5" t="s" s="2">
         <v>36</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E5" t="s" s="2">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@f5e0636831eee57a3be155238bf6af26cadf174f 🚀
</commit_message>
<xml_diff>
--- a/epic-rolcode.xlsx
+++ b/epic-rolcode.xlsx
@@ -42,7 +42,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Epic qualifier &amp; role to SNOMED-CT Mapping</t>
+    <t>Epic Practitioner Type naar SNOMED-CT Mapping</t>
   </si>
   <si>
     <t>Status</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-07-22T09:30:07+00:00</t>
+    <t>2024-07-22T09:39:12+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -87,7 +87,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Deze ConceptMap representeert de mapping tussen de Epic Practitioner.qualifier SER#6000 naar een SNOMED-CT code.</t>
+    <t>Deze ConceptMap representeert de mapping tussen Epic Practitioner Type naar een SNOMED-CT code.</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@5853bac8191bb2ed98eea45d518ff9a57b6e6005 🚀
</commit_message>
<xml_diff>
--- a/epic-rolcode.xlsx
+++ b/epic-rolcode.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-07-22T09:39:12+00:00</t>
+    <t>2024-07-22T09:54:11+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -108,7 +108,7 @@
     <t>Target</t>
   </si>
   <si>
-    <t>urn:oid:1.2.840.114350.1.13.485.3.7.10.836982.1040</t>
+    <t>urn:oid:1.2.840.114350.1.13.485.3.7.10.836982.1040|UMCG Epic</t>
   </si>
   <si>
     <t/>

</xml_diff>